<commit_message>
feat(daily-pickup): 엑셀 다운로드를 OTA+G-OTA 기준으로 변경
- build_excel(seg_label) 추가, main에서 OTA+G-OTA 행만 필터해 엑셀 생성(요약·일별·누적·상세)
- 엑셀 제목/§6/주석에 'OTA+G-OTA 기준' 명시, 합계 10,624/11,247/-623 (화면 기본뷰 동일)
- JSON은 전 세그 보존(화면 필터용), 페이지 주석 갱신

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/RM_FCST_정리.xlsx
+++ b/data/RM_FCST_정리.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="사업장별 총괄" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="세그먼트별 상세" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="메타정보" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사업장별 총괄" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="세그먼트별 상세" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="메타정보" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
chore(gs-weekly): 8월 마지막주 → 9월 뷰 전환
WEEK_VIEW_OVERRIDE=true + rm_fcst_view_override.txt=2026-09. 당월 9월 RM FCST=67,916 /
누계 1~9월=673,145. 정적 PPT/xlsx 9월(GS otb_data 9월 객실+소사업). 롤오버 시 원복.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/RM_FCST_정리.xlsx
+++ b/data/RM_FCST_정리.xlsx
@@ -478,7 +478,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>RM FCST - 2026-08</t>
+          <t>RM FCST - 2026-09</t>
         </is>
       </c>
     </row>
@@ -541,31 +541,31 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>35550</v>
+        <v>17100</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>193</v>
+        <v>141</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>6866</v>
+        <v>2410</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>30942</v>
+        <v>15870</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>211</v>
+        <v>162</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>6544</v>
+        <v>2566</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>87</v>
+        <v>92.8</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>97.40000000000001</v>
+        <v>96.3</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>6641.4</v>
+        <v>2662.3</v>
       </c>
     </row>
     <row r="4">
@@ -575,31 +575,31 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>6265</v>
+        <v>3420</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>280</v>
+        <v>244</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>1757</v>
+        <v>833</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>7907</v>
+        <v>3091</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>264</v>
+        <v>226</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>2086</v>
+        <v>700</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>126.2</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>33.3</v>
+        <v>20.4</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>2119.3</v>
+        <v>720.4</v>
       </c>
     </row>
     <row r="5">
@@ -609,31 +609,31 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>3837</v>
+        <v>2210</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>375</v>
+        <v>340</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>1440</v>
+        <v>752</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>3320</v>
+        <v>2074</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>391</v>
+        <v>341</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>1298</v>
+        <v>708</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>86.5</v>
+        <v>93.8</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>10.4</v>
+        <v>14</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>1308.4</v>
+        <v>722</v>
       </c>
     </row>
     <row r="6">
@@ -643,31 +643,31 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>8955</v>
+        <v>4500</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>320</v>
+        <v>264</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>2866</v>
+        <v>1188</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>7612</v>
+        <v>4305</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>334</v>
+        <v>292</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>2546</v>
+        <v>1257</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>85</v>
+        <v>95.7</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>14</v>
+        <v>17.5</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>2560</v>
+        <v>1274.5</v>
       </c>
     </row>
     <row r="7">
@@ -677,31 +677,31 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>4382</v>
+        <v>2732</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>363</v>
+        <v>308</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>1592</v>
+        <v>841</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>3879</v>
+        <v>2651</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>384</v>
+        <v>329</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>1488</v>
+        <v>872</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>88.5</v>
+        <v>97</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>7.3</v>
+        <v>10.2</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>1495.3</v>
+        <v>882.2</v>
       </c>
     </row>
     <row r="8">
@@ -711,31 +711,31 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>4010</v>
+        <v>3355</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>151</v>
+        <v>128</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>607</v>
+        <v>430</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>3294</v>
+        <v>2913</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>166</v>
+        <v>140</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>548</v>
+        <v>409</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>82.09999999999999</v>
+        <v>86.8</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>549.5</v>
+        <v>410.7</v>
       </c>
     </row>
     <row r="9">
@@ -745,31 +745,31 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>32350</v>
+        <v>20345</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>244</v>
+        <v>218</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>7888</v>
+        <v>4445</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>32780</v>
+        <v>19051</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>244</v>
+        <v>230</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>7998</v>
+        <v>4390</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>101.3</v>
+        <v>93.59999999999999</v>
       </c>
       <c r="I9" s="4" t="n">
-        <v>104</v>
+        <v>123.2</v>
       </c>
       <c r="J9" s="4" t="n">
-        <v>8102</v>
+        <v>4513.2</v>
       </c>
     </row>
     <row r="10">
@@ -779,31 +779,31 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>15180</v>
+        <v>10645</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>229</v>
+        <v>181</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>3477</v>
+        <v>1924</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>14792</v>
+        <v>9120</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>235</v>
+        <v>194</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>3478</v>
+        <v>1768</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>97.40000000000001</v>
+        <v>85.7</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>32.2</v>
+        <v>35.3</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>3510.2</v>
+        <v>1803.3</v>
       </c>
     </row>
     <row r="11">
@@ -813,31 +813,31 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>21305</v>
+        <v>17890</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>248</v>
+        <v>208</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>5282</v>
+        <v>3730</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>21500</v>
+        <v>16350</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>247</v>
+        <v>211</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>5304</v>
+        <v>3452</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>100.9</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="I11" s="4" t="n">
-        <v>101.4</v>
+        <v>63.3</v>
       </c>
       <c r="J11" s="4" t="n">
-        <v>5405.4</v>
+        <v>3515.3</v>
       </c>
     </row>
     <row r="12">
@@ -847,31 +847,31 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>18300</v>
+        <v>12830</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>187</v>
+        <v>160</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>3424</v>
+        <v>2051</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>17200</v>
+        <v>10580</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>197</v>
+        <v>177</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>3380</v>
+        <v>1872</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>94</v>
+        <v>82.5</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>215.4</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>3595.4</v>
+        <v>1952.4</v>
       </c>
     </row>
     <row r="13">
@@ -881,31 +881,31 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>11100</v>
+        <v>9195</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>259</v>
+        <v>229</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>2876</v>
+        <v>2109</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>12610</v>
+        <v>10350</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>274</v>
+        <v>234</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>3461</v>
+        <v>2423</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>113.6</v>
+        <v>112.6</v>
       </c>
       <c r="I13" s="4" t="n">
-        <v>56</v>
+        <v>44.9</v>
       </c>
       <c r="J13" s="4" t="n">
-        <v>3517</v>
+        <v>2467.9</v>
       </c>
     </row>
     <row r="14">
@@ -915,31 +915,31 @@
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>5545</v>
+        <v>4250</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>192</v>
+        <v>155</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>1066</v>
+        <v>657</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>5440</v>
+        <v>4360</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>200</v>
+        <v>173</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>1089</v>
+        <v>754</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>98.09999999999999</v>
+        <v>102.6</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>10.3</v>
+        <v>18.8</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>1099.3</v>
+        <v>772.8</v>
       </c>
     </row>
     <row r="15">
@@ -949,31 +949,31 @@
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>12590</v>
+        <v>7800</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>202</v>
+        <v>164</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>2548</v>
+        <v>1280</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>12463</v>
+        <v>7586</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>212</v>
+        <v>177</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>2642</v>
+        <v>1341</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>99</v>
+        <v>97.3</v>
       </c>
       <c r="I15" s="4" t="n">
-        <v>205.4</v>
+        <v>105.5</v>
       </c>
       <c r="J15" s="4" t="n">
-        <v>2847.4</v>
+        <v>1446.5</v>
       </c>
     </row>
     <row r="16">
@@ -983,31 +983,31 @@
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>13660</v>
+        <v>9000</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>194</v>
+        <v>160</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>2657</v>
+        <v>1444</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>13840</v>
+        <v>7821</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>196</v>
+        <v>176</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>2715</v>
+        <v>1379</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>101.3</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="I16" s="4" t="n">
-        <v>196.2</v>
+        <v>113.2</v>
       </c>
       <c r="J16" s="4" t="n">
-        <v>2911.2</v>
+        <v>1492.2</v>
       </c>
     </row>
     <row r="17">
@@ -1017,31 +1017,31 @@
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>6190</v>
+        <v>4860</v>
       </c>
       <c r="C17" s="3" t="n">
-        <v>300</v>
+        <v>248</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>1858</v>
+        <v>1204</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>5795</v>
+        <v>4500</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>300</v>
+        <v>262</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>1737</v>
+        <v>1179</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>93.59999999999999</v>
+        <v>92.59999999999999</v>
       </c>
       <c r="I17" s="4" t="n">
-        <v>65.90000000000001</v>
+        <v>54.8</v>
       </c>
       <c r="J17" s="4" t="n">
-        <v>1802.9</v>
+        <v>1233.8</v>
       </c>
     </row>
     <row r="18">
@@ -1051,31 +1051,31 @@
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>14120</v>
+        <v>8570</v>
       </c>
       <c r="C18" s="3" t="n">
-        <v>262</v>
+        <v>206</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>3700</v>
+        <v>1769</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>13455</v>
+        <v>7050</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>267</v>
+        <v>229</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>3596</v>
+        <v>1614</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>95.3</v>
+        <v>82.3</v>
       </c>
       <c r="I18" s="4" t="n">
-        <v>62.9</v>
+        <v>97.3</v>
       </c>
       <c r="J18" s="4" t="n">
-        <v>3658.9</v>
+        <v>1711.3</v>
       </c>
     </row>
     <row r="19">
@@ -1085,31 +1085,31 @@
         </is>
       </c>
       <c r="B19" s="3" t="n">
-        <v>16710</v>
+        <v>10970</v>
       </c>
       <c r="C19" s="3" t="n">
-        <v>248</v>
+        <v>198</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>4149</v>
+        <v>2176</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>15010</v>
+        <v>8375</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>258</v>
+        <v>218</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>3873</v>
+        <v>1828</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>89.8</v>
+        <v>76.3</v>
       </c>
       <c r="I19" s="4" t="n">
-        <v>59.6</v>
+        <v>28.5</v>
       </c>
       <c r="J19" s="4" t="n">
-        <v>3932.6</v>
+        <v>1856.5</v>
       </c>
     </row>
     <row r="20">
@@ -1119,31 +1119,31 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>10130</v>
+        <v>9160</v>
       </c>
       <c r="C20" s="3" t="n">
-        <v>204</v>
+        <v>165</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>2063</v>
+        <v>1515</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>10080</v>
+        <v>9320</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>219</v>
+        <v>169</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>2210</v>
+        <v>1574</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>99.5</v>
+        <v>101.7</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>13.6</v>
+        <v>11.3</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>2223.6</v>
+        <v>1585.3</v>
       </c>
     </row>
     <row r="21">
@@ -1153,31 +1153,31 @@
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>6280</v>
+        <v>6920</v>
       </c>
       <c r="C21" s="3" t="n">
-        <v>247</v>
+        <v>203</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>1549</v>
+        <v>1404</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>6970</v>
+        <v>6340</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>242</v>
+        <v>201</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>1690</v>
+        <v>1272</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>111</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="I21" s="4" t="n">
-        <v>40.5</v>
+        <v>27.9</v>
       </c>
       <c r="J21" s="4" t="n">
-        <v>1730.5</v>
+        <v>1299.9</v>
       </c>
     </row>
     <row r="22">
@@ -1187,31 +1187,31 @@
         </is>
       </c>
       <c r="B22" s="3" t="n">
-        <v>16100</v>
+        <v>15350</v>
       </c>
       <c r="C22" s="3" t="n">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>2257</v>
+        <v>2094</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>13988</v>
+        <v>14460</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>158</v>
+        <v>149</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>2207</v>
+        <v>2158</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>86.90000000000001</v>
+        <v>94.2</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>113</v>
+        <v>133.5</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>2320</v>
+        <v>2291.5</v>
       </c>
     </row>
     <row r="23">
@@ -1221,31 +1221,31 @@
         </is>
       </c>
       <c r="B23" s="3" t="n">
-        <v>6470</v>
+        <v>5845</v>
       </c>
       <c r="C23" s="3" t="n">
-        <v>137</v>
+        <v>98</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>884</v>
+        <v>572</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>6622</v>
+        <v>5500</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>151</v>
+        <v>98</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>1002</v>
+        <v>538</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>102.3</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="I23" s="4" t="n">
-        <v>74.90000000000001</v>
+        <v>22.9</v>
       </c>
       <c r="J23" s="4" t="n">
-        <v>1076.9</v>
+        <v>560.9</v>
       </c>
     </row>
     <row r="24">
@@ -1255,31 +1255,31 @@
         </is>
       </c>
       <c r="B24" s="3" t="n">
-        <v>12300</v>
+        <v>11080</v>
       </c>
       <c r="C24" s="3" t="n">
-        <v>365</v>
+        <v>312</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>4493</v>
+        <v>3451</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>12746</v>
+        <v>8405</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>364</v>
+        <v>323</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>4639</v>
+        <v>2717</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>103.6</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="I24" s="4" t="n">
-        <v>26.5</v>
+        <v>7.9</v>
       </c>
       <c r="J24" s="4" t="n">
-        <v>4665.5</v>
+        <v>2724.9</v>
       </c>
     </row>
     <row r="25">
@@ -1289,31 +1289,31 @@
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>2455</v>
+        <v>2150</v>
       </c>
       <c r="C25" s="3" t="n">
-        <v>366</v>
+        <v>252</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>898</v>
+        <v>542</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>2575</v>
+        <v>2000</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>367</v>
+        <v>251</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>945</v>
+        <v>503</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>104.9</v>
+        <v>93</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>17.4</v>
+        <v>12.8</v>
       </c>
       <c r="J25" s="4" t="n">
-        <v>962.4</v>
+        <v>515.8</v>
       </c>
     </row>
     <row r="26">
@@ -1323,13 +1323,13 @@
         </is>
       </c>
       <c r="G26" s="6" t="n">
-        <v>66476</v>
+        <v>37274</v>
       </c>
       <c r="I26" s="7" t="n">
-        <v>1559.1</v>
+        <v>1141.6</v>
       </c>
       <c r="J26" s="7" t="n">
-        <v>68035.10000000001</v>
+        <v>38415.6</v>
       </c>
     </row>
     <row r="27"/>
@@ -1340,25 +1340,25 @@
         </is>
       </c>
       <c r="B28" s="6" t="n">
-        <v>62999</v>
+        <v>33317</v>
       </c>
       <c r="C28" s="6" t="n">
-        <v>240</v>
+        <v>194</v>
       </c>
       <c r="D28" s="6" t="n">
-        <v>15128</v>
+        <v>6453</v>
       </c>
       <c r="E28" s="6" t="n">
-        <v>56954</v>
+        <v>30904</v>
       </c>
       <c r="F28" s="6" t="n">
-        <v>255</v>
+        <v>211</v>
       </c>
       <c r="G28" s="6" t="n">
-        <v>14511</v>
+        <v>6512</v>
       </c>
       <c r="H28" s="7" t="n">
-        <v>90.40000000000001</v>
+        <v>92.8</v>
       </c>
     </row>
     <row r="29">
@@ -1368,25 +1368,25 @@
         </is>
       </c>
       <c r="B29" s="6" t="n">
-        <v>102180</v>
+        <v>71660</v>
       </c>
       <c r="C29" s="6" t="n">
-        <v>230</v>
+        <v>195</v>
       </c>
       <c r="D29" s="6" t="n">
-        <v>23517</v>
+        <v>13972</v>
       </c>
       <c r="E29" s="6" t="n">
-        <v>101310</v>
+        <v>64687</v>
       </c>
       <c r="F29" s="6" t="n">
-        <v>234</v>
+        <v>206</v>
       </c>
       <c r="G29" s="6" t="n">
-        <v>23747</v>
+        <v>13326</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>99.09999999999999</v>
+        <v>90.3</v>
       </c>
     </row>
     <row r="30">
@@ -1396,25 +1396,25 @@
         </is>
       </c>
       <c r="B30" s="6" t="n">
-        <v>32510</v>
+        <v>31430</v>
       </c>
       <c r="C30" s="6" t="n">
-        <v>181</v>
+        <v>160</v>
       </c>
       <c r="D30" s="6" t="n">
-        <v>5869</v>
+        <v>5013</v>
       </c>
       <c r="E30" s="6" t="n">
-        <v>31038</v>
+        <v>30120</v>
       </c>
       <c r="F30" s="6" t="n">
-        <v>197</v>
+        <v>166</v>
       </c>
       <c r="G30" s="6" t="n">
-        <v>6107</v>
+        <v>5004</v>
       </c>
       <c r="H30" s="7" t="n">
-        <v>95.5</v>
+        <v>95.8</v>
       </c>
     </row>
     <row r="31">
@@ -1424,25 +1424,25 @@
         </is>
       </c>
       <c r="B31" s="6" t="n">
-        <v>86095</v>
+        <v>63770</v>
       </c>
       <c r="C31" s="6" t="n">
-        <v>252</v>
+        <v>210</v>
       </c>
       <c r="D31" s="6" t="n">
-        <v>21681</v>
+        <v>13382</v>
       </c>
       <c r="E31" s="6" t="n">
-        <v>85518</v>
+        <v>56361</v>
       </c>
       <c r="F31" s="6" t="n">
-        <v>259</v>
+        <v>221</v>
       </c>
       <c r="G31" s="6" t="n">
-        <v>22111</v>
+        <v>12432</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>99.3</v>
+        <v>88.40000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -1468,7 +1468,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>RM FCST 세그먼트별 - 2026-08</t>
+          <t>RM FCST 세그먼트별 - 2026-09</t>
         </is>
       </c>
     </row>
@@ -1546,34 +1546,34 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>11500</v>
+        <v>4350</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>205</v>
+        <v>159</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>2358</v>
+        <v>692</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>9350</v>
+        <v>3850</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>237</v>
+        <v>174</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>2220</v>
+        <v>670</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>81.3</v>
+        <v>88.5</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>-2150</v>
+        <v>-500</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>8.300000000000001</v>
+        <v>15.6</v>
       </c>
       <c r="L3" s="4" t="n">
-        <v>78</v>
+        <v>60.1</v>
       </c>
     </row>
     <row r="4">
@@ -1588,34 +1588,34 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>2800</v>
+        <v>1500</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>205</v>
+        <v>157</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>574</v>
+        <v>236</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>3170</v>
+        <v>1350</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>243</v>
+        <v>190</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>770</v>
+        <v>257</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>113.2</v>
+        <v>90</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>370</v>
+        <v>-150</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>5.2</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>16.3</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="5">
@@ -1630,34 +1630,34 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>145</v>
+        <v>82</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>43</v>
+        <v>16</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>68</v>
+        <v>680</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>8</v>
+        <v>74</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>22.7</v>
+        <v>340</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>-232</v>
+        <v>480</v>
       </c>
       <c r="K5" s="4" t="n">
-        <v>45.6</v>
+        <v>34.9</v>
       </c>
       <c r="L5" s="4" t="n">
-        <v>3.1</v>
+        <v>23.7</v>
       </c>
     </row>
     <row r="6">
@@ -1672,34 +1672,34 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>2060</v>
+        <v>920</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>297</v>
+        <v>251</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>612</v>
+        <v>231</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>3440</v>
+        <v>880</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>273</v>
+        <v>235</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>939</v>
+        <v>207</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>167</v>
+        <v>95.7</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>1380</v>
+        <v>-40</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>8.300000000000001</v>
+        <v>15.6</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>28.7</v>
+        <v>13.7</v>
       </c>
     </row>
     <row r="7">
@@ -1714,34 +1714,34 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>1010</v>
+        <v>710</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>300</v>
+        <v>263</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>303</v>
+        <v>187</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>900</v>
+        <v>370</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>292</v>
+        <v>267</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>262</v>
+        <v>99</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>89.09999999999999</v>
+        <v>52.1</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>-110</v>
+        <v>-340</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>5.2</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="L7" s="4" t="n">
-        <v>4.6</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="8">
@@ -1765,25 +1765,25 @@
         <v>0</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>0</v>
+        <v>92</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>0</v>
+        <v>178</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="I8" s="4" t="n">
         <v>0</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>0</v>
+        <v>92</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>45.6</v>
+        <v>34.9</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>0</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="9">
@@ -1798,34 +1798,34 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>1150</v>
+        <v>650</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>369</v>
+        <v>360</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>424</v>
+        <v>234</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>780</v>
+        <v>600</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>417</v>
+        <v>343</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>326</v>
+        <v>206</v>
       </c>
       <c r="I9" s="4" t="n">
-        <v>67.8</v>
+        <v>92.3</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>-370</v>
+        <v>-50</v>
       </c>
       <c r="K9" s="4" t="n">
-        <v>8.300000000000001</v>
+        <v>15.6</v>
       </c>
       <c r="L9" s="4" t="n">
-        <v>6.5</v>
+        <v>9.4</v>
       </c>
     </row>
     <row r="10">
@@ -1840,34 +1840,34 @@
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>950</v>
+        <v>400</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>400</v>
+        <v>350</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>380</v>
+        <v>140</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>755</v>
+        <v>500</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>408</v>
+        <v>345</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>308</v>
+        <v>173</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>79.5</v>
+        <v>125</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>-195</v>
+        <v>100</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>5.2</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>3.9</v>
+        <v>4.6</v>
       </c>
     </row>
     <row r="11">
@@ -1906,7 +1906,7 @@
         <v>0</v>
       </c>
       <c r="K11" s="4" t="n">
-        <v>45.6</v>
+        <v>34.9</v>
       </c>
       <c r="L11" s="4" t="n">
         <v>0</v>
@@ -1924,34 +1924,34 @@
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>2400</v>
+        <v>950</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>347</v>
+        <v>280</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>833</v>
+        <v>266</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>1920</v>
+        <v>956</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>373</v>
+        <v>309</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>716</v>
+        <v>295</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>80</v>
+        <v>100.6</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>-480</v>
+        <v>6</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>4.8</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>9.199999999999999</v>
+        <v>8.800000000000001</v>
       </c>
     </row>
     <row r="13">
@@ -1966,34 +1966,34 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>1600</v>
+        <v>700</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>344</v>
+        <v>284</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>550</v>
+        <v>199</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>1360</v>
+        <v>750</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>362</v>
+        <v>303</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>493</v>
+        <v>227</v>
       </c>
       <c r="I13" s="4" t="n">
-        <v>85</v>
+        <v>107.1</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>-240</v>
+        <v>50</v>
       </c>
       <c r="K13" s="4" t="n">
-        <v>3.5</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="L13" s="4" t="n">
-        <v>4.8</v>
+        <v>7.3</v>
       </c>
     </row>
     <row r="14">
@@ -2017,25 +2017,25 @@
         <v>0</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>0</v>
+        <v>216</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I14" s="4" t="n">
         <v>0</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K14" s="4" t="n">
         <v>468.4</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>0</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="15">
@@ -2050,34 +2050,34 @@
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>1150</v>
+        <v>600</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>392</v>
+        <v>340</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>451</v>
+        <v>204</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>1140</v>
+        <v>700</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>423</v>
+        <v>354</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>482</v>
+        <v>248</v>
       </c>
       <c r="I15" s="4" t="n">
-        <v>99.09999999999999</v>
+        <v>116.7</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>-10</v>
+        <v>100</v>
       </c>
       <c r="K15" s="4" t="n">
-        <v>4.8</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="L15" s="4" t="n">
-        <v>5.5</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="16">
@@ -2092,34 +2092,34 @@
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>700</v>
+        <v>420</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>380</v>
+        <v>336</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>266</v>
+        <v>141</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>530</v>
+        <v>385</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>404</v>
+        <v>338</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>214</v>
+        <v>130</v>
       </c>
       <c r="I16" s="4" t="n">
-        <v>75.7</v>
+        <v>91.7</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>-170</v>
+        <v>-35</v>
       </c>
       <c r="K16" s="4" t="n">
-        <v>3.5</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="L16" s="4" t="n">
-        <v>1.9</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="17">
@@ -2179,31 +2179,31 @@
         <v>450</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>183</v>
+        <v>167</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>390</v>
+        <v>380</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>214</v>
+        <v>171</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="I18" s="4" t="n">
-        <v>86.7</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>-60</v>
+        <v>-70</v>
       </c>
       <c r="K18" s="4" t="n">
-        <v>3.2</v>
+        <v>2.1</v>
       </c>
       <c r="L18" s="4" t="n">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="19">
@@ -2218,34 +2218,34 @@
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>315</v>
+        <v>300</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>350</v>
+        <v>330</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>194</v>
+        <v>165</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>68</v>
+        <v>54</v>
       </c>
       <c r="I19" s="4" t="n">
-        <v>111.1</v>
+        <v>110</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="K19" s="4" t="n">
-        <v>0.7</v>
+        <v>0.1</v>
       </c>
       <c r="L19" s="4" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -2260,34 +2260,34 @@
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>0</v>
+        <v>68</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I20" s="4" t="n">
         <v>0</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>-20</v>
+        <v>30</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>3.6</v>
+        <v>29.3</v>
       </c>
       <c r="L20" s="4" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="21">
@@ -2302,34 +2302,34 @@
         </is>
       </c>
       <c r="C21" s="3" t="n">
-        <v>5610</v>
+        <v>3750</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>288</v>
+        <v>269</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>1613</v>
+        <v>1009</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>5650</v>
+        <v>4000</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>294</v>
+        <v>272</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>1661</v>
+        <v>1088</v>
       </c>
       <c r="I21" s="4" t="n">
-        <v>100.7</v>
+        <v>106.7</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>40</v>
+        <v>250</v>
       </c>
       <c r="K21" s="4" t="n">
-        <v>12.6</v>
+        <v>25.2</v>
       </c>
       <c r="L21" s="4" t="n">
-        <v>71.09999999999999</v>
+        <v>100.6</v>
       </c>
     </row>
     <row r="22">
@@ -2344,34 +2344,34 @@
         </is>
       </c>
       <c r="C22" s="3" t="n">
-        <v>3700</v>
+        <v>2900</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>250</v>
+        <v>225</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>925</v>
+        <v>652</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>4400</v>
+        <v>3100</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>263</v>
+        <v>247</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>1159</v>
+        <v>766</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>118.9</v>
+        <v>106.9</v>
       </c>
       <c r="J22" s="3" t="n">
-        <v>700</v>
+        <v>200</v>
       </c>
       <c r="K22" s="4" t="n">
-        <v>7.3</v>
+        <v>7</v>
       </c>
       <c r="L22" s="4" t="n">
-        <v>32.1</v>
+        <v>21.6</v>
       </c>
     </row>
     <row r="23">
@@ -2386,34 +2386,34 @@
         </is>
       </c>
       <c r="C23" s="3" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>117</v>
+        <v>95</v>
       </c>
       <c r="E23" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F23" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="G23" s="3" t="n">
+        <v>80</v>
+      </c>
+      <c r="H23" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="F23" s="3" t="n">
-        <v>31</v>
-      </c>
-      <c r="G23" s="3" t="n">
-        <v>147</v>
-      </c>
-      <c r="H23" s="3" t="n">
-        <v>5</v>
-      </c>
       <c r="I23" s="4" t="n">
-        <v>155</v>
+        <v>48</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>11</v>
+        <v>-26</v>
       </c>
       <c r="K23" s="4" t="n">
-        <v>24.8</v>
+        <v>39</v>
       </c>
       <c r="L23" s="4" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="24">
@@ -2428,34 +2428,34 @@
         </is>
       </c>
       <c r="C24" s="3" t="n">
-        <v>2050</v>
+        <v>1650</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>264</v>
+        <v>194</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>542</v>
+        <v>320</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>1990</v>
+        <v>1550</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>277</v>
+        <v>210</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>550</v>
+        <v>326</v>
       </c>
       <c r="I24" s="4" t="n">
-        <v>97.09999999999999</v>
+        <v>93.90000000000001</v>
       </c>
       <c r="J24" s="3" t="n">
-        <v>-60</v>
+        <v>-100</v>
       </c>
       <c r="K24" s="4" t="n">
-        <v>9.800000000000001</v>
+        <v>13.3</v>
       </c>
       <c r="L24" s="4" t="n">
-        <v>19.4</v>
+        <v>20.5</v>
       </c>
     </row>
     <row r="25">
@@ -2470,34 +2470,34 @@
         </is>
       </c>
       <c r="C25" s="3" t="n">
-        <v>1200</v>
+        <v>1550</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>225</v>
+        <v>182</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>270</v>
+        <v>282</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>1500</v>
+        <v>1350</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>235</v>
+        <v>196</v>
       </c>
       <c r="H25" s="3" t="n">
-        <v>353</v>
+        <v>265</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>125</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="J25" s="3" t="n">
-        <v>300</v>
+        <v>-200</v>
       </c>
       <c r="K25" s="4" t="n">
-        <v>8.5</v>
+        <v>11</v>
       </c>
       <c r="L25" s="4" t="n">
-        <v>12.8</v>
+        <v>14.8</v>
       </c>
     </row>
     <row r="26">
@@ -2536,7 +2536,7 @@
         <v>0</v>
       </c>
       <c r="K26" s="4" t="n">
-        <v>90.90000000000001</v>
+        <v>0</v>
       </c>
       <c r="L26" s="4" t="n">
         <v>0</v>
@@ -2554,34 +2554,34 @@
         </is>
       </c>
       <c r="C27" s="3" t="n">
-        <v>3000</v>
+        <v>3600</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>282</v>
+        <v>222</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>846</v>
+        <v>799</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>2960</v>
+        <v>3450</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>291</v>
+        <v>230</v>
       </c>
       <c r="H27" s="3" t="n">
-        <v>861</v>
+        <v>794</v>
       </c>
       <c r="I27" s="4" t="n">
-        <v>98.7</v>
+        <v>95.8</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>-40</v>
+        <v>-150</v>
       </c>
       <c r="K27" s="4" t="n">
-        <v>17.1</v>
+        <v>12.8</v>
       </c>
       <c r="L27" s="4" t="n">
-        <v>50.7</v>
+        <v>44.1</v>
       </c>
     </row>
     <row r="28">
@@ -2596,34 +2596,34 @@
         </is>
       </c>
       <c r="C28" s="3" t="n">
-        <v>1400</v>
+        <v>2400</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>280</v>
+        <v>215</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>392</v>
+        <v>516</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>1821</v>
+        <v>2450</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>268</v>
+        <v>222</v>
       </c>
       <c r="H28" s="3" t="n">
-        <v>488</v>
+        <v>544</v>
       </c>
       <c r="I28" s="4" t="n">
-        <v>130.1</v>
+        <v>102.1</v>
       </c>
       <c r="J28" s="3" t="n">
-        <v>421</v>
+        <v>50</v>
       </c>
       <c r="K28" s="4" t="n">
-        <v>27.8</v>
+        <v>7.8</v>
       </c>
       <c r="L28" s="4" t="n">
-        <v>50.7</v>
+        <v>19.2</v>
       </c>
     </row>
     <row r="29">
@@ -2680,34 +2680,34 @@
         </is>
       </c>
       <c r="C30" s="3" t="n">
-        <v>5150</v>
+        <v>3700</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>198</v>
+        <v>176</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>1018</v>
+        <v>652</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>5365</v>
+        <v>2500</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>221</v>
+        <v>202</v>
       </c>
       <c r="H30" s="3" t="n">
-        <v>1186</v>
+        <v>504</v>
       </c>
       <c r="I30" s="4" t="n">
-        <v>104.2</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="J30" s="3" t="n">
-        <v>215</v>
+        <v>-1200</v>
       </c>
       <c r="K30" s="4" t="n">
-        <v>30.4</v>
+        <v>22.6</v>
       </c>
       <c r="L30" s="4" t="n">
-        <v>163.2</v>
+        <v>56.4</v>
       </c>
     </row>
     <row r="31">
@@ -2722,34 +2722,34 @@
         </is>
       </c>
       <c r="C31" s="3" t="n">
-        <v>3000</v>
+        <v>2050</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>189</v>
+        <v>172</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>568</v>
+        <v>353</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>3215</v>
+        <v>1850</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>667</v>
+        <v>362</v>
       </c>
       <c r="I31" s="4" t="n">
-        <v>107.2</v>
+        <v>90.2</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>215</v>
+        <v>-200</v>
       </c>
       <c r="K31" s="4" t="n">
-        <v>15.9</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="L31" s="4" t="n">
-        <v>51.1</v>
+        <v>18.1</v>
       </c>
     </row>
     <row r="32">
@@ -2764,34 +2764,34 @@
         </is>
       </c>
       <c r="C32" s="3" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>101</v>
+        <v>78</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>50</v>
+        <v>140</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>93</v>
+        <v>65</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="I32" s="4" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="J32" s="3" t="n">
-        <v>-50</v>
+        <v>-60</v>
       </c>
       <c r="K32" s="4" t="n">
-        <v>22.6</v>
+        <v>42.5</v>
       </c>
       <c r="L32" s="4" t="n">
-        <v>1.1</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="33">
@@ -2806,34 +2806,34 @@
         </is>
       </c>
       <c r="C33" s="3" t="n">
-        <v>1725</v>
+        <v>1460</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>301</v>
+        <v>265</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>520</v>
+        <v>387</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>2620</v>
+        <v>2100</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>339</v>
+        <v>270</v>
       </c>
       <c r="H33" s="3" t="n">
-        <v>888</v>
+        <v>567</v>
       </c>
       <c r="I33" s="4" t="n">
-        <v>151.9</v>
+        <v>143.8</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>895</v>
+        <v>640</v>
       </c>
       <c r="K33" s="4" t="n">
         <v>19.2</v>
       </c>
       <c r="L33" s="4" t="n">
-        <v>50.4</v>
+        <v>40.4</v>
       </c>
     </row>
     <row r="34">
@@ -2848,34 +2848,34 @@
         </is>
       </c>
       <c r="C34" s="3" t="n">
-        <v>1165</v>
+        <v>970</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>302</v>
+        <v>267</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>352</v>
+        <v>259</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>1600</v>
+        <v>1250</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>314</v>
+        <v>247</v>
       </c>
       <c r="H34" s="3" t="n">
-        <v>502</v>
+        <v>309</v>
       </c>
       <c r="I34" s="4" t="n">
-        <v>137.3</v>
+        <v>128.9</v>
       </c>
       <c r="J34" s="3" t="n">
-        <v>435</v>
+        <v>280</v>
       </c>
       <c r="K34" s="4" t="n">
         <v>3.5</v>
       </c>
       <c r="L34" s="4" t="n">
-        <v>5.6</v>
+        <v>4.4</v>
       </c>
     </row>
     <row r="35">
@@ -2899,10 +2899,10 @@
         <v>0</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>0</v>
+        <v>236</v>
       </c>
       <c r="H35" s="3" t="n">
         <v>0</v>
@@ -2911,13 +2911,13 @@
         <v>0</v>
       </c>
       <c r="J35" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K35" s="4" t="n">
         <v>51.9</v>
       </c>
       <c r="L35" s="4" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="36">
@@ -2932,34 +2932,34 @@
         </is>
       </c>
       <c r="C36" s="3" t="n">
-        <v>1175</v>
+        <v>985</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>202</v>
+        <v>167</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>237</v>
+        <v>165</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>1125</v>
+        <v>1050</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>232</v>
+        <v>196</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>261</v>
+        <v>206</v>
       </c>
       <c r="I36" s="4" t="n">
-        <v>95.7</v>
+        <v>106.6</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>-50</v>
+        <v>65</v>
       </c>
       <c r="K36" s="4" t="n">
-        <v>6.6</v>
+        <v>9.6</v>
       </c>
       <c r="L36" s="4" t="n">
-        <v>7.4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="37">
@@ -2974,34 +2974,34 @@
         </is>
       </c>
       <c r="C37" s="3" t="n">
+        <v>600</v>
+      </c>
+      <c r="D37" s="3" t="n">
+        <v>154</v>
+      </c>
+      <c r="E37" s="3" t="n">
+        <v>93</v>
+      </c>
+      <c r="F37" s="3" t="n">
         <v>730</v>
       </c>
-      <c r="D37" s="3" t="n">
-        <v>198</v>
-      </c>
-      <c r="E37" s="3" t="n">
-        <v>145</v>
-      </c>
-      <c r="F37" s="3" t="n">
-        <v>880</v>
-      </c>
       <c r="G37" s="3" t="n">
-        <v>232</v>
+        <v>185</v>
       </c>
       <c r="H37" s="3" t="n">
-        <v>204</v>
+        <v>135</v>
       </c>
       <c r="I37" s="4" t="n">
-        <v>120.5</v>
+        <v>121.7</v>
       </c>
       <c r="J37" s="3" t="n">
-        <v>150</v>
+        <v>130</v>
       </c>
       <c r="K37" s="4" t="n">
-        <v>3</v>
+        <v>11.4</v>
       </c>
       <c r="L37" s="4" t="n">
-        <v>2.6</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="38">
@@ -3016,34 +3016,34 @@
         </is>
       </c>
       <c r="C38" s="3" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="D38" s="3" t="n">
-        <v>237</v>
+        <v>0</v>
       </c>
       <c r="E38" s="3" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="H38" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I38" s="4" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="J38" s="3" t="n">
-        <v>-14</v>
+        <v>10</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>42.4</v>
+        <v>45.4</v>
       </c>
       <c r="L38" s="4" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="39">
@@ -3058,34 +3058,34 @@
         </is>
       </c>
       <c r="C39" s="3" t="n">
-        <v>3450</v>
+        <v>1650</v>
       </c>
       <c r="D39" s="3" t="n">
-        <v>208</v>
+        <v>187</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>719</v>
+        <v>309</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>3570</v>
+        <v>1900</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>221</v>
+        <v>194</v>
       </c>
       <c r="H39" s="3" t="n">
-        <v>788</v>
+        <v>368</v>
       </c>
       <c r="I39" s="4" t="n">
-        <v>103.5</v>
+        <v>115.2</v>
       </c>
       <c r="J39" s="3" t="n">
-        <v>120</v>
+        <v>250</v>
       </c>
       <c r="K39" s="4" t="n">
         <v>43.9</v>
       </c>
       <c r="L39" s="4" t="n">
-        <v>156.6</v>
+        <v>83.40000000000001</v>
       </c>
     </row>
     <row r="40">
@@ -3100,34 +3100,34 @@
         </is>
       </c>
       <c r="C40" s="3" t="n">
-        <v>1500</v>
+        <v>950</v>
       </c>
       <c r="D40" s="3" t="n">
-        <v>204</v>
+        <v>187</v>
       </c>
       <c r="E40" s="3" t="n">
-        <v>306</v>
+        <v>178</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>2090</v>
+        <v>950</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>214</v>
+        <v>195</v>
       </c>
       <c r="H40" s="3" t="n">
-        <v>447</v>
+        <v>185</v>
       </c>
       <c r="I40" s="4" t="n">
-        <v>139.3</v>
+        <v>100</v>
       </c>
       <c r="J40" s="3" t="n">
-        <v>590</v>
+        <v>0</v>
       </c>
       <c r="K40" s="4" t="n">
         <v>23.4</v>
       </c>
       <c r="L40" s="4" t="n">
-        <v>48.8</v>
+        <v>22.2</v>
       </c>
     </row>
     <row r="41">
@@ -3184,34 +3184,34 @@
         </is>
       </c>
       <c r="C42" s="3" t="n">
-        <v>2600</v>
+        <v>1500</v>
       </c>
       <c r="D42" s="3" t="n">
-        <v>222</v>
+        <v>180</v>
       </c>
       <c r="E42" s="3" t="n">
-        <v>577</v>
+        <v>269</v>
       </c>
       <c r="F42" s="3" t="n">
-        <v>2527</v>
+        <v>1500</v>
       </c>
       <c r="G42" s="3" t="n">
-        <v>225</v>
+        <v>192</v>
       </c>
       <c r="H42" s="3" t="n">
-        <v>568</v>
+        <v>288</v>
       </c>
       <c r="I42" s="4" t="n">
-        <v>97.2</v>
+        <v>100</v>
       </c>
       <c r="J42" s="3" t="n">
-        <v>-73</v>
+        <v>0</v>
       </c>
       <c r="K42" s="4" t="n">
-        <v>62.5</v>
+        <v>50.1</v>
       </c>
       <c r="L42" s="4" t="n">
-        <v>158</v>
+        <v>75.09999999999999</v>
       </c>
     </row>
     <row r="43">
@@ -3226,34 +3226,34 @@
         </is>
       </c>
       <c r="C43" s="3" t="n">
-        <v>1450</v>
+        <v>1000</v>
       </c>
       <c r="D43" s="3" t="n">
-        <v>207</v>
+        <v>168</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>300</v>
+        <v>168</v>
       </c>
       <c r="F43" s="3" t="n">
-        <v>1490</v>
+        <v>900</v>
       </c>
       <c r="G43" s="3" t="n">
-        <v>201</v>
+        <v>188</v>
       </c>
       <c r="H43" s="3" t="n">
-        <v>300</v>
+        <v>169</v>
       </c>
       <c r="I43" s="4" t="n">
-        <v>102.8</v>
+        <v>90</v>
       </c>
       <c r="J43" s="3" t="n">
-        <v>40</v>
+        <v>-100</v>
       </c>
       <c r="K43" s="4" t="n">
-        <v>25.7</v>
+        <v>16.7</v>
       </c>
       <c r="L43" s="4" t="n">
-        <v>38.2</v>
+        <v>15.1</v>
       </c>
     </row>
     <row r="44">
@@ -3277,25 +3277,25 @@
         <v>0</v>
       </c>
       <c r="F44" s="3" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="G44" s="3" t="n">
-        <v>0</v>
+        <v>133</v>
       </c>
       <c r="H44" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I44" s="4" t="n">
         <v>0</v>
       </c>
       <c r="J44" s="3" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="K44" s="4" t="n">
-        <v>23.6</v>
+        <v>1440</v>
       </c>
       <c r="L44" s="4" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
     </row>
     <row r="45">
@@ -3310,34 +3310,34 @@
         </is>
       </c>
       <c r="C45" s="3" t="n">
-        <v>750</v>
+        <v>500</v>
       </c>
       <c r="D45" s="3" t="n">
-        <v>333</v>
+        <v>266</v>
       </c>
       <c r="E45" s="3" t="n">
-        <v>250</v>
+        <v>133</v>
       </c>
       <c r="F45" s="3" t="n">
-        <v>480</v>
+        <v>400</v>
       </c>
       <c r="G45" s="3" t="n">
-        <v>365</v>
+        <v>288</v>
       </c>
       <c r="H45" s="3" t="n">
-        <v>175</v>
+        <v>115</v>
       </c>
       <c r="I45" s="4" t="n">
-        <v>64</v>
+        <v>80</v>
       </c>
       <c r="J45" s="3" t="n">
-        <v>-270</v>
+        <v>-100</v>
       </c>
       <c r="K45" s="4" t="n">
-        <v>79.7</v>
+        <v>60.3</v>
       </c>
       <c r="L45" s="4" t="n">
-        <v>38.3</v>
+        <v>24.1</v>
       </c>
     </row>
     <row r="46">
@@ -3352,34 +3352,34 @@
         </is>
       </c>
       <c r="C46" s="3" t="n">
-        <v>1000</v>
+        <v>700</v>
       </c>
       <c r="D46" s="3" t="n">
-        <v>333</v>
+        <v>256</v>
       </c>
       <c r="E46" s="3" t="n">
-        <v>333</v>
+        <v>179</v>
       </c>
       <c r="F46" s="3" t="n">
-        <v>1100</v>
+        <v>800</v>
       </c>
       <c r="G46" s="3" t="n">
-        <v>343</v>
+        <v>275</v>
       </c>
       <c r="H46" s="3" t="n">
-        <v>378</v>
+        <v>220</v>
       </c>
       <c r="I46" s="4" t="n">
-        <v>110</v>
+        <v>114.3</v>
       </c>
       <c r="J46" s="3" t="n">
         <v>100</v>
       </c>
       <c r="K46" s="4" t="n">
-        <v>24.2</v>
+        <v>38</v>
       </c>
       <c r="L46" s="4" t="n">
-        <v>26.6</v>
+        <v>30.4</v>
       </c>
     </row>
     <row r="47">
@@ -3394,34 +3394,34 @@
         </is>
       </c>
       <c r="C47" s="3" t="n">
-        <v>0</v>
+        <v>190</v>
       </c>
       <c r="D47" s="3" t="n">
-        <v>0</v>
+        <v>145</v>
       </c>
       <c r="E47" s="3" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="F47" s="3" t="n">
-        <v>31</v>
+        <v>89</v>
       </c>
       <c r="G47" s="3" t="n">
-        <v>177</v>
+        <v>154</v>
       </c>
       <c r="H47" s="3" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="I47" s="4" t="n">
-        <v>0</v>
+        <v>46.8</v>
       </c>
       <c r="J47" s="3" t="n">
-        <v>31</v>
+        <v>-101</v>
       </c>
       <c r="K47" s="4" t="n">
-        <v>34</v>
+        <v>2.6</v>
       </c>
       <c r="L47" s="4" t="n">
-        <v>1.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="48">
@@ -3436,34 +3436,34 @@
         </is>
       </c>
       <c r="C48" s="3" t="n">
-        <v>2400</v>
+        <v>1300</v>
       </c>
       <c r="D48" s="3" t="n">
-        <v>285</v>
+        <v>235</v>
       </c>
       <c r="E48" s="3" t="n">
-        <v>684</v>
+        <v>306</v>
       </c>
       <c r="F48" s="3" t="n">
-        <v>2900</v>
+        <v>1250</v>
       </c>
       <c r="G48" s="3" t="n">
-        <v>313</v>
+        <v>260</v>
       </c>
       <c r="H48" s="3" t="n">
-        <v>906</v>
+        <v>325</v>
       </c>
       <c r="I48" s="4" t="n">
-        <v>120.8</v>
+        <v>96.2</v>
       </c>
       <c r="J48" s="3" t="n">
-        <v>500</v>
+        <v>-50</v>
       </c>
       <c r="K48" s="4" t="n">
-        <v>13.2</v>
+        <v>43.2</v>
       </c>
       <c r="L48" s="4" t="n">
-        <v>38.4</v>
+        <v>53.9</v>
       </c>
     </row>
     <row r="49">
@@ -3478,34 +3478,34 @@
         </is>
       </c>
       <c r="C49" s="3" t="n">
-        <v>1750</v>
+        <v>1020</v>
       </c>
       <c r="D49" s="3" t="n">
-        <v>279</v>
+        <v>234</v>
       </c>
       <c r="E49" s="3" t="n">
-        <v>488</v>
+        <v>239</v>
       </c>
       <c r="F49" s="3" t="n">
-        <v>1730</v>
+        <v>1350</v>
       </c>
       <c r="G49" s="3" t="n">
-        <v>288</v>
+        <v>235</v>
       </c>
       <c r="H49" s="3" t="n">
-        <v>499</v>
+        <v>318</v>
       </c>
       <c r="I49" s="4" t="n">
-        <v>98.90000000000001</v>
+        <v>132.4</v>
       </c>
       <c r="J49" s="3" t="n">
-        <v>-20</v>
+        <v>330</v>
       </c>
       <c r="K49" s="4" t="n">
-        <v>14.2</v>
+        <v>31.9</v>
       </c>
       <c r="L49" s="4" t="n">
-        <v>24.6</v>
+        <v>43.1</v>
       </c>
     </row>
     <row r="50">
@@ -3529,25 +3529,25 @@
         <v>0</v>
       </c>
       <c r="F50" s="3" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G50" s="3" t="n">
-        <v>0</v>
+        <v>222</v>
       </c>
       <c r="H50" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I50" s="4" t="n">
         <v>0</v>
       </c>
       <c r="J50" s="3" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K50" s="4" t="n">
-        <v>35.9</v>
+        <v>27.3</v>
       </c>
       <c r="L50" s="4" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="51">
@@ -3562,34 +3562,34 @@
         </is>
       </c>
       <c r="C51" s="3" t="n">
-        <v>3300</v>
+        <v>2500</v>
       </c>
       <c r="D51" s="3" t="n">
-        <v>270</v>
+        <v>217</v>
       </c>
       <c r="E51" s="3" t="n">
-        <v>891</v>
+        <v>543</v>
       </c>
       <c r="F51" s="3" t="n">
-        <v>3045</v>
+        <v>2000</v>
       </c>
       <c r="G51" s="3" t="n">
-        <v>294</v>
+        <v>232</v>
       </c>
       <c r="H51" s="3" t="n">
-        <v>896</v>
+        <v>464</v>
       </c>
       <c r="I51" s="4" t="n">
-        <v>92.3</v>
+        <v>80</v>
       </c>
       <c r="J51" s="3" t="n">
-        <v>-255</v>
+        <v>-500</v>
       </c>
       <c r="K51" s="4" t="n">
-        <v>11.3</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="L51" s="4" t="n">
-        <v>34.3</v>
+        <v>16.4</v>
       </c>
     </row>
     <row r="52">
@@ -3604,34 +3604,34 @@
         </is>
       </c>
       <c r="C52" s="3" t="n">
-        <v>2600</v>
+        <v>1500</v>
       </c>
       <c r="D52" s="3" t="n">
-        <v>262</v>
+        <v>199</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>680</v>
+        <v>299</v>
       </c>
       <c r="F52" s="3" t="n">
-        <v>2280</v>
+        <v>1570</v>
       </c>
       <c r="G52" s="3" t="n">
-        <v>279</v>
+        <v>220</v>
       </c>
       <c r="H52" s="3" t="n">
-        <v>636</v>
+        <v>346</v>
       </c>
       <c r="I52" s="4" t="n">
-        <v>87.7</v>
+        <v>104.7</v>
       </c>
       <c r="J52" s="3" t="n">
-        <v>-320</v>
+        <v>70</v>
       </c>
       <c r="K52" s="4" t="n">
-        <v>11.1</v>
+        <v>7.7</v>
       </c>
       <c r="L52" s="4" t="n">
-        <v>25.3</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="53">
@@ -3670,7 +3670,7 @@
         <v>0</v>
       </c>
       <c r="K53" s="4" t="n">
-        <v>0</v>
+        <v>37.8</v>
       </c>
       <c r="L53" s="4" t="n">
         <v>0</v>
@@ -3688,34 +3688,34 @@
         </is>
       </c>
       <c r="C54" s="3" t="n">
-        <v>1200</v>
+        <v>900</v>
       </c>
       <c r="D54" s="3" t="n">
-        <v>214</v>
+        <v>184</v>
       </c>
       <c r="E54" s="3" t="n">
-        <v>257</v>
+        <v>166</v>
       </c>
       <c r="F54" s="3" t="n">
-        <v>1170</v>
+        <v>900</v>
       </c>
       <c r="G54" s="3" t="n">
-        <v>273</v>
+        <v>193</v>
       </c>
       <c r="H54" s="3" t="n">
-        <v>320</v>
+        <v>174</v>
       </c>
       <c r="I54" s="4" t="n">
-        <v>97.5</v>
+        <v>100</v>
       </c>
       <c r="J54" s="3" t="n">
-        <v>-30</v>
+        <v>0</v>
       </c>
       <c r="K54" s="4" t="n">
-        <v>6.8</v>
+        <v>5.7</v>
       </c>
       <c r="L54" s="4" t="n">
-        <v>7.9</v>
+        <v>5.1</v>
       </c>
     </row>
     <row r="55">
@@ -3730,34 +3730,34 @@
         </is>
       </c>
       <c r="C55" s="3" t="n">
-        <v>2300</v>
+        <v>1550</v>
       </c>
       <c r="D55" s="3" t="n">
-        <v>210</v>
+        <v>177</v>
       </c>
       <c r="E55" s="3" t="n">
-        <v>483</v>
+        <v>274</v>
       </c>
       <c r="F55" s="3" t="n">
-        <v>2060</v>
+        <v>1650</v>
       </c>
       <c r="G55" s="3" t="n">
-        <v>235</v>
+        <v>169</v>
       </c>
       <c r="H55" s="3" t="n">
-        <v>484</v>
+        <v>279</v>
       </c>
       <c r="I55" s="4" t="n">
-        <v>89.59999999999999</v>
+        <v>106.5</v>
       </c>
       <c r="J55" s="3" t="n">
-        <v>-240</v>
+        <v>100</v>
       </c>
       <c r="K55" s="4" t="n">
-        <v>2.5</v>
+        <v>2.9</v>
       </c>
       <c r="L55" s="4" t="n">
-        <v>5.2</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="56">
@@ -3772,34 +3772,34 @@
         </is>
       </c>
       <c r="C56" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D56" s="3" t="n">
-        <v>0</v>
+        <v>63</v>
       </c>
       <c r="E56" s="3" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F56" s="3" t="n">
-        <v>17</v>
+        <v>55</v>
       </c>
       <c r="G56" s="3" t="n">
         <v>73</v>
       </c>
       <c r="H56" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I56" s="4" t="n">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="J56" s="3" t="n">
-        <v>17</v>
+        <v>-45</v>
       </c>
       <c r="K56" s="4" t="n">
         <v>23.8</v>
       </c>
       <c r="L56" s="4" t="n">
-        <v>0.4</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="57">
@@ -3814,34 +3814,34 @@
         </is>
       </c>
       <c r="C57" s="3" t="n">
-        <v>570</v>
+        <v>650</v>
       </c>
       <c r="D57" s="3" t="n">
-        <v>293</v>
+        <v>250</v>
       </c>
       <c r="E57" s="3" t="n">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="F57" s="3" t="n">
-        <v>815</v>
+        <v>670</v>
       </c>
       <c r="G57" s="3" t="n">
-        <v>288</v>
+        <v>235</v>
       </c>
       <c r="H57" s="3" t="n">
-        <v>235</v>
+        <v>157</v>
       </c>
       <c r="I57" s="4" t="n">
-        <v>143</v>
+        <v>103.1</v>
       </c>
       <c r="J57" s="3" t="n">
-        <v>245</v>
+        <v>20</v>
       </c>
       <c r="K57" s="4" t="n">
-        <v>24.7</v>
+        <v>19.2</v>
       </c>
       <c r="L57" s="4" t="n">
-        <v>20.1</v>
+        <v>12.9</v>
       </c>
     </row>
     <row r="58">
@@ -3856,34 +3856,34 @@
         </is>
       </c>
       <c r="C58" s="3" t="n">
-        <v>680</v>
+        <v>710</v>
       </c>
       <c r="D58" s="3" t="n">
-        <v>284</v>
+        <v>245</v>
       </c>
       <c r="E58" s="3" t="n">
-        <v>193</v>
+        <v>174</v>
       </c>
       <c r="F58" s="3" t="n">
-        <v>1075</v>
+        <v>790</v>
       </c>
       <c r="G58" s="3" t="n">
-        <v>260</v>
+        <v>222</v>
       </c>
       <c r="H58" s="3" t="n">
-        <v>280</v>
+        <v>175</v>
       </c>
       <c r="I58" s="4" t="n">
-        <v>158.1</v>
+        <v>111.3</v>
       </c>
       <c r="J58" s="3" t="n">
-        <v>395</v>
+        <v>80</v>
       </c>
       <c r="K58" s="4" t="n">
-        <v>18.9</v>
+        <v>19</v>
       </c>
       <c r="L58" s="4" t="n">
-        <v>20.4</v>
+        <v>15</v>
       </c>
     </row>
     <row r="59">
@@ -3907,19 +3907,19 @@
         <v>0</v>
       </c>
       <c r="F59" s="3" t="n">
-        <v>0</v>
+        <v>67</v>
       </c>
       <c r="G59" s="3" t="n">
-        <v>0</v>
+        <v>178</v>
       </c>
       <c r="H59" s="3" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="I59" s="4" t="n">
         <v>0</v>
       </c>
       <c r="J59" s="3" t="n">
-        <v>0</v>
+        <v>67</v>
       </c>
       <c r="K59" s="4" t="n">
         <v>0</v>
@@ -3940,34 +3940,34 @@
         </is>
       </c>
       <c r="C60" s="3" t="n">
-        <v>1700</v>
+        <v>1400</v>
       </c>
       <c r="D60" s="3" t="n">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="E60" s="3" t="n">
-        <v>322</v>
+        <v>260</v>
       </c>
       <c r="F60" s="3" t="n">
-        <v>1050</v>
+        <v>1000</v>
       </c>
       <c r="G60" s="3" t="n">
-        <v>245</v>
+        <v>200</v>
       </c>
       <c r="H60" s="3" t="n">
-        <v>257</v>
+        <v>200</v>
       </c>
       <c r="I60" s="4" t="n">
-        <v>61.8</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="J60" s="3" t="n">
-        <v>-650</v>
+        <v>-400</v>
       </c>
       <c r="K60" s="4" t="n">
-        <v>14.3</v>
+        <v>17.3</v>
       </c>
       <c r="L60" s="4" t="n">
-        <v>15</v>
+        <v>17.3</v>
       </c>
     </row>
     <row r="61">
@@ -3982,34 +3982,34 @@
         </is>
       </c>
       <c r="C61" s="3" t="n">
-        <v>2500</v>
+        <v>2800</v>
       </c>
       <c r="D61" s="3" t="n">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="E61" s="3" t="n">
-        <v>471</v>
+        <v>515</v>
       </c>
       <c r="F61" s="3" t="n">
-        <v>2350</v>
+        <v>2850</v>
       </c>
       <c r="G61" s="3" t="n">
-        <v>219</v>
+        <v>200</v>
       </c>
       <c r="H61" s="3" t="n">
-        <v>516</v>
+        <v>570</v>
       </c>
       <c r="I61" s="4" t="n">
-        <v>94</v>
+        <v>101.8</v>
       </c>
       <c r="J61" s="3" t="n">
-        <v>-150</v>
+        <v>50</v>
       </c>
       <c r="K61" s="4" t="n">
-        <v>1.2</v>
+        <v>2.1</v>
       </c>
       <c r="L61" s="4" t="n">
-        <v>2.7</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="62">
@@ -4033,25 +4033,25 @@
         <v>276</v>
       </c>
       <c r="F62" s="3" t="n">
-        <v>2420</v>
+        <v>3000</v>
       </c>
       <c r="G62" s="3" t="n">
+        <v>95</v>
+      </c>
+      <c r="H62" s="3" t="n">
+        <v>285</v>
+      </c>
+      <c r="I62" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="H62" s="3" t="n">
-        <v>241</v>
-      </c>
-      <c r="I62" s="4" t="n">
-        <v>80.7</v>
-      </c>
       <c r="J62" s="3" t="n">
-        <v>-580</v>
+        <v>0</v>
       </c>
       <c r="K62" s="4" t="n">
-        <v>39.4</v>
+        <v>36.7</v>
       </c>
       <c r="L62" s="4" t="n">
-        <v>95.3</v>
+        <v>110</v>
       </c>
     </row>
     <row r="63">
@@ -4066,34 +4066,34 @@
         </is>
       </c>
       <c r="C63" s="3" t="n">
-        <v>800</v>
+        <v>700</v>
       </c>
       <c r="D63" s="3" t="n">
-        <v>133</v>
+        <v>96</v>
       </c>
       <c r="E63" s="3" t="n">
-        <v>106</v>
+        <v>67</v>
       </c>
       <c r="F63" s="3" t="n">
-        <v>550</v>
+        <v>430</v>
       </c>
       <c r="G63" s="3" t="n">
-        <v>178</v>
+        <v>105</v>
       </c>
       <c r="H63" s="3" t="n">
-        <v>98</v>
+        <v>45</v>
       </c>
       <c r="I63" s="4" t="n">
-        <v>68.8</v>
+        <v>61.4</v>
       </c>
       <c r="J63" s="3" t="n">
-        <v>-250</v>
+        <v>-270</v>
       </c>
       <c r="K63" s="4" t="n">
-        <v>37.1</v>
+        <v>30.8</v>
       </c>
       <c r="L63" s="4" t="n">
-        <v>20.4</v>
+        <v>13.2</v>
       </c>
     </row>
     <row r="64">
@@ -4108,34 +4108,34 @@
         </is>
       </c>
       <c r="C64" s="3" t="n">
-        <v>1500</v>
+        <v>1100</v>
       </c>
       <c r="D64" s="3" t="n">
-        <v>133</v>
+        <v>93</v>
       </c>
       <c r="E64" s="3" t="n">
-        <v>200</v>
+        <v>102</v>
       </c>
       <c r="F64" s="3" t="n">
-        <v>1790</v>
+        <v>1400</v>
       </c>
       <c r="G64" s="3" t="n">
-        <v>162</v>
+        <v>96</v>
       </c>
       <c r="H64" s="3" t="n">
-        <v>291</v>
+        <v>134</v>
       </c>
       <c r="I64" s="4" t="n">
-        <v>119.3</v>
+        <v>127.3</v>
       </c>
       <c r="J64" s="3" t="n">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="K64" s="4" t="n">
-        <v>8.1</v>
+        <v>4.7</v>
       </c>
       <c r="L64" s="4" t="n">
-        <v>14.4</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="65">
@@ -4150,34 +4150,34 @@
         </is>
       </c>
       <c r="C65" s="3" t="n">
-        <v>700</v>
+        <v>800</v>
       </c>
       <c r="D65" s="3" t="n">
-        <v>87</v>
+        <v>70</v>
       </c>
       <c r="E65" s="3" t="n">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="F65" s="3" t="n">
-        <v>1325</v>
+        <v>1002</v>
       </c>
       <c r="G65" s="3" t="n">
-        <v>92</v>
+        <v>74</v>
       </c>
       <c r="H65" s="3" t="n">
-        <v>122</v>
+        <v>74</v>
       </c>
       <c r="I65" s="4" t="n">
-        <v>189.3</v>
+        <v>125.2</v>
       </c>
       <c r="J65" s="3" t="n">
-        <v>625</v>
+        <v>202</v>
       </c>
       <c r="K65" s="4" t="n">
-        <v>30.2</v>
+        <v>3</v>
       </c>
       <c r="L65" s="4" t="n">
-        <v>40.1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="66">
@@ -4192,34 +4192,34 @@
         </is>
       </c>
       <c r="C66" s="3" t="n">
-        <v>1860</v>
+        <v>1780</v>
       </c>
       <c r="D66" s="3" t="n">
-        <v>425</v>
+        <v>358</v>
       </c>
       <c r="E66" s="3" t="n">
-        <v>791</v>
+        <v>637</v>
       </c>
       <c r="F66" s="3" t="n">
-        <v>2380</v>
+        <v>1500</v>
       </c>
       <c r="G66" s="3" t="n">
-        <v>409</v>
+        <v>343</v>
       </c>
       <c r="H66" s="3" t="n">
-        <v>972</v>
+        <v>515</v>
       </c>
       <c r="I66" s="4" t="n">
-        <v>128</v>
+        <v>84.3</v>
       </c>
       <c r="J66" s="3" t="n">
-        <v>520</v>
+        <v>-280</v>
       </c>
       <c r="K66" s="4" t="n">
-        <v>1.8</v>
+        <v>1.1</v>
       </c>
       <c r="L66" s="4" t="n">
-        <v>4.4</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="67">
@@ -4234,34 +4234,34 @@
         </is>
       </c>
       <c r="C67" s="3" t="n">
-        <v>980</v>
+        <v>970</v>
       </c>
       <c r="D67" s="3" t="n">
-        <v>421</v>
+        <v>361</v>
       </c>
       <c r="E67" s="3" t="n">
-        <v>413</v>
+        <v>350</v>
       </c>
       <c r="F67" s="3" t="n">
-        <v>1640</v>
+        <v>1400</v>
       </c>
       <c r="G67" s="3" t="n">
-        <v>398</v>
+        <v>348</v>
       </c>
       <c r="H67" s="3" t="n">
-        <v>652</v>
+        <v>487</v>
       </c>
       <c r="I67" s="4" t="n">
-        <v>167.3</v>
+        <v>144.3</v>
       </c>
       <c r="J67" s="3" t="n">
-        <v>660</v>
+        <v>430</v>
       </c>
       <c r="K67" s="4" t="n">
-        <v>13.5</v>
+        <v>4.4</v>
       </c>
       <c r="L67" s="4" t="n">
-        <v>22.1</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="68">
@@ -4318,34 +4318,34 @@
         </is>
       </c>
       <c r="C69" s="3" t="n">
-        <v>800</v>
+        <v>500</v>
       </c>
       <c r="D69" s="3" t="n">
-        <v>380</v>
+        <v>273</v>
       </c>
       <c r="E69" s="3" t="n">
-        <v>304</v>
+        <v>137</v>
       </c>
       <c r="F69" s="3" t="n">
-        <v>925</v>
+        <v>600</v>
       </c>
       <c r="G69" s="3" t="n">
-        <v>356</v>
+        <v>252</v>
       </c>
       <c r="H69" s="3" t="n">
-        <v>329</v>
+        <v>151</v>
       </c>
       <c r="I69" s="4" t="n">
-        <v>115.6</v>
+        <v>120</v>
       </c>
       <c r="J69" s="3" t="n">
-        <v>125</v>
+        <v>100</v>
       </c>
       <c r="K69" s="4" t="n">
         <v>13.5</v>
       </c>
       <c r="L69" s="4" t="n">
-        <v>12.5</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="70">
@@ -4360,34 +4360,34 @@
         </is>
       </c>
       <c r="C70" s="3" t="n">
-        <v>550</v>
+        <v>355</v>
       </c>
       <c r="D70" s="3" t="n">
-        <v>381</v>
+        <v>272</v>
       </c>
       <c r="E70" s="3" t="n">
-        <v>210</v>
+        <v>97</v>
       </c>
       <c r="F70" s="3" t="n">
-        <v>480</v>
+        <v>455</v>
       </c>
       <c r="G70" s="3" t="n">
-        <v>335</v>
+        <v>217</v>
       </c>
       <c r="H70" s="3" t="n">
-        <v>161</v>
+        <v>99</v>
       </c>
       <c r="I70" s="4" t="n">
-        <v>87.3</v>
+        <v>128.2</v>
       </c>
       <c r="J70" s="3" t="n">
-        <v>-70</v>
+        <v>100</v>
       </c>
       <c r="K70" s="4" t="n">
         <v>10.2</v>
       </c>
       <c r="L70" s="4" t="n">
-        <v>4.9</v>
+        <v>4.6</v>
       </c>
     </row>
     <row r="71">
@@ -4494,7 +4494,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-09</t>
         </is>
       </c>
     </row>
@@ -4518,7 +4518,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>전년 2025-08 실당소사업 × FCST 객실수 (미운영 사업장은 2026-05 대체)</t>
+          <t>전년 2025-09 실당소사업 × FCST 객실수 (미운영 사업장은 2026-05 대체)</t>
         </is>
       </c>
     </row>

</xml_diff>